<commit_message>
Add points for 3hsg9oklerq6uua8pos3dmdck_playerlog
</commit_message>
<xml_diff>
--- a/bnc-streamlit-app/data/points/3hsg9oklerq6uua8pos3dmdck_playerlog.xlsx
+++ b/bnc-streamlit-app/data/points/3hsg9oklerq6uua8pos3dmdck_playerlog.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BG30"/>
+  <dimension ref="A1:BG32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -780,14 +780,14 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="n">
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
@@ -835,7 +835,7 @@
         <v>0</v>
       </c>
       <c r="AM2" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="AN2" t="n">
         <v>0</v>
@@ -955,14 +955,14 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="n">
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
@@ -1008,21 +1008,21 @@
         </is>
       </c>
       <c r="AI3" t="n">
-        <v>-0.4801966500000001</v>
+        <v>-0.5193438400000001</v>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>-1.09</t>
+          <t>-1.11</t>
         </is>
       </c>
       <c r="AK3" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="AL3" t="n">
         <v>0</v>
       </c>
       <c r="AM3" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="AN3" t="n">
         <v>0</v>
@@ -1142,14 +1142,14 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="n">
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="S4" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
@@ -1195,7 +1195,7 @@
         </is>
       </c>
       <c r="AI4" t="n">
-        <v>1.2753758</v>
+        <v>1.2622772</v>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
@@ -1209,7 +1209,7 @@
         <v>0</v>
       </c>
       <c r="AM4" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="AN4" t="n">
         <v>0</v>
@@ -1227,7 +1227,7 @@
         <v>6</v>
       </c>
       <c r="AS4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT4" t="n">
         <v>1</v>
@@ -1396,11 +1396,11 @@
         </is>
       </c>
       <c r="AI5" t="n">
-        <v>2.47944565</v>
+        <v>2.47717292</v>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>+1.87</t>
+          <t>+1.89</t>
         </is>
       </c>
       <c r="AK5" t="n">
@@ -1526,14 +1526,14 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="n">
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -1541,7 +1541,7 @@
         </is>
       </c>
       <c r="S6" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>+0.58</t>
+          <t>+0.60</t>
         </is>
       </c>
       <c r="AK6" t="n">
@@ -1593,7 +1593,7 @@
         <v>0</v>
       </c>
       <c r="AM6" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="AN6" t="n">
         <v>0</v>
@@ -1713,14 +1713,14 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="n">
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
@@ -1728,7 +1728,7 @@
         </is>
       </c>
       <c r="S7" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
@@ -1766,11 +1766,11 @@
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>1.94744842</v>
+        <v>1.9951514</v>
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>+1.34</t>
+          <t>+1.41</t>
         </is>
       </c>
       <c r="AK7" t="n">
@@ -1780,7 +1780,7 @@
         <v>0</v>
       </c>
       <c r="AM7" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="AN7" t="n">
         <v>0</v>
@@ -1798,7 +1798,7 @@
         <v>3</v>
       </c>
       <c r="AS7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AT7" t="n">
         <v>2</v>
@@ -1836,7 +1836,7 @@
         </is>
       </c>
       <c r="BE7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="BF7" t="n">
         <v>2</v>
@@ -1886,10 +1886,12 @@
           <t>72m84nwa6dshu3ibmy13dz5rd</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
+      <c r="I8" t="n">
+        <v>2</v>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
@@ -1900,7 +1902,7 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1911,7 +1913,7 @@
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -1935,7 +1937,7 @@
         </is>
       </c>
       <c r="W8" t="n">
-        <v>29.8</v>
+        <v>31.8</v>
       </c>
       <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr"/>
@@ -1961,7 +1963,7 @@
         <v>-0.05</v>
       </c>
       <c r="AG8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
@@ -1969,30 +1971,30 @@
         </is>
       </c>
       <c r="AI8" t="n">
-        <v>1.31017453</v>
+        <v>1.91017453</v>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>+0.70</t>
+          <t>+1.32</t>
         </is>
       </c>
       <c r="AK8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AL8" t="n">
         <v>0</v>
       </c>
       <c r="AM8" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AN8" t="n">
         <v>0</v>
       </c>
       <c r="AO8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AQ8" t="n">
         <v>0</v>
@@ -2042,10 +2044,10 @@
         <v>9</v>
       </c>
       <c r="BF8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BG8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -2162,7 +2164,7 @@
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>+0.13</t>
+          <t>+0.15</t>
         </is>
       </c>
       <c r="AK9" t="n">
@@ -2347,7 +2349,7 @@
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>-0.27</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="AK10" t="n">
@@ -2477,7 +2479,7 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -2488,7 +2490,7 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -2504,7 +2506,7 @@
         </is>
       </c>
       <c r="U11" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
@@ -2540,21 +2542,21 @@
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>1.32379127</v>
+        <v>1.37067553</v>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>+0.72</t>
+          <t>+0.78</t>
         </is>
       </c>
       <c r="AK11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AL11" t="n">
         <v>0</v>
       </c>
       <c r="AM11" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="AN11" t="n">
         <v>0</v>
@@ -2572,13 +2574,13 @@
         <v>3</v>
       </c>
       <c r="AS11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT11" t="n">
         <v>0</v>
       </c>
       <c r="AU11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AV11" t="n">
         <v>0</v>
@@ -2670,7 +2672,7 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -2681,7 +2683,7 @@
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -2697,7 +2699,7 @@
         </is>
       </c>
       <c r="U12" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
@@ -2737,17 +2739,17 @@
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>+1.04</t>
+          <t>+1.05</t>
         </is>
       </c>
       <c r="AK12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AL12" t="n">
         <v>0</v>
       </c>
       <c r="AM12" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="AN12" t="n">
         <v>0</v>
@@ -2871,14 +2873,14 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="n">
         <v>92</v>
       </c>
       <c r="Q13" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
@@ -2886,7 +2888,7 @@
         </is>
       </c>
       <c r="S13" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
@@ -2924,11 +2926,11 @@
         </is>
       </c>
       <c r="AI13" t="n">
-        <v>0.0985451</v>
+        <v>0.12709712</v>
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
-          <t>-0.51</t>
+          <t>-0.46</t>
         </is>
       </c>
       <c r="AK13" t="n">
@@ -2938,7 +2940,7 @@
         <v>92</v>
       </c>
       <c r="AM13" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="AN13" t="n">
         <v>0</v>
@@ -2956,7 +2958,7 @@
         <v>0</v>
       </c>
       <c r="AS13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT13" t="n">
         <v>0</v>
@@ -3012,17 +3014,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Endrick</t>
+          <t>Danilo Santos</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 19</t>
+          <t xml:space="preserve"> 18</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>RCM(3)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -3037,7 +3039,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>14qv8npo5alwnb5dud8x82ln8</t>
+          <t>dsvi49wsvjqdbiddyme3xow7o</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
@@ -3047,7 +3049,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>45</v>
+        <v>97</v>
       </c>
       <c r="L14" t="n">
         <v>2</v>
@@ -3058,22 +3060,22 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>50</v>
+        <v>3</v>
       </c>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="n">
-        <v>45</v>
+        <v>97</v>
       </c>
       <c r="Q14" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>RCM(3)</t>
         </is>
       </c>
       <c r="S14" t="n">
-        <v>50</v>
+        <v>3</v>
       </c>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
@@ -3094,38 +3096,38 @@
         </is>
       </c>
       <c r="AD14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AE14" t="n">
         <v>0</v>
       </c>
       <c r="AF14" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AG14" t="n">
         <v>2</v>
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>Endrick</t>
+          <t>Danilo Santos</t>
         </is>
       </c>
       <c r="AI14" t="n">
-        <v>0.04598741000000001</v>
+        <v>0</v>
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
-          <t>-0.56</t>
+          <t>-0.59</t>
         </is>
       </c>
       <c r="AK14" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="AL14" t="n">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="AM14" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="AN14" t="n">
         <v>0</v>
@@ -3140,7 +3142,7 @@
         <v>0</v>
       </c>
       <c r="AR14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AS14" t="n">
         <v>0</v>
@@ -3199,12 +3201,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Gabriel Martinelli</t>
+          <t>Endrick</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 22</t>
+          <t xml:space="preserve"> 19</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -3224,7 +3226,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>7ocm7nugzwos59il1pm4eub8q</t>
+          <t>14qv8npo5alwnb5dud8x82ln8</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
@@ -3234,7 +3236,7 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="L15" t="n">
         <v>2</v>
@@ -3245,18 +3247,14 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>30</v>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>LCM(2)</t>
-        </is>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="O15" t="inlineStr"/>
       <c r="P15" t="n">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="Q15" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
@@ -3264,16 +3262,10 @@
         </is>
       </c>
       <c r="S15" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>LCM(2)</t>
-        </is>
-      </c>
-      <c r="U15" t="n">
-        <v>29.8</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr"/>
       <c r="X15" t="inlineStr"/>
@@ -3291,7 +3283,7 @@
         </is>
       </c>
       <c r="AD15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE15" t="n">
         <v>0</v>
@@ -3304,43 +3296,43 @@
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>Gabriel Martinelli</t>
+          <t>Endrick</t>
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>1.40653567</v>
+        <v>0.09598741000000001</v>
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t>+0.80</t>
+          <t>-0.49</t>
         </is>
       </c>
       <c r="AK15" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="AL15" t="n">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="AM15" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="AN15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO15" t="n">
         <v>0</v>
       </c>
       <c r="AP15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ15" t="n">
         <v>0</v>
       </c>
       <c r="AR15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AS15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT15" t="n">
         <v>0</v>
@@ -3352,7 +3344,7 @@
         <v>0</v>
       </c>
       <c r="AW15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX15" t="n">
         <v>0</v>
@@ -3377,7 +3369,7 @@
         <v>0</v>
       </c>
       <c r="BF15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BG15" t="n">
         <v>0</v>
@@ -3391,37 +3383,37 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>6duaxcbrofil112qfq4v895go</t>
+          <t>ajab3nmpoltsoeqcuoyi4pwzx</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Z. Suzuki</t>
+          <t>Gabriel Martinelli</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t xml:space="preserve"> 22</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>GK</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2mfunwzltzdnmzlcjyvx752i</t>
+          <t>7ocm7nugzwos59il1pm4eub8q</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
@@ -3430,33 +3422,47 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
+      <c r="K16" t="n">
+        <v>65</v>
+      </c>
+      <c r="L16" t="n">
+        <v>2</v>
+      </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N16" t="n">
-        <v>95</v>
-      </c>
-      <c r="O16" t="inlineStr"/>
+        <v>35</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>LCM(2)</t>
+        </is>
+      </c>
       <c r="P16" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="Q16" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>GK</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="S16" t="n">
-        <v>95</v>
-      </c>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr"/>
+        <v>0.2</v>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>LCM(2)</t>
+        </is>
+      </c>
+      <c r="U16" t="n">
+        <v>34.8</v>
+      </c>
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr"/>
       <c r="X16" t="inlineStr"/>
@@ -3465,50 +3471,62 @@
       <c r="AA16" t="inlineStr"/>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>6duaxcbrofil112qfq4v895go</t>
+          <t>ajab3nmpoltsoeqcuoyi4pwzx</t>
         </is>
       </c>
       <c r="AC16" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="AD16" t="n">
         <v>1</v>
       </c>
       <c r="AE16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AF16" t="n">
         <v>0</v>
       </c>
       <c r="AG16" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH16" t="inlineStr"/>
-      <c r="AI16" t="inlineStr"/>
-      <c r="AJ16" t="inlineStr"/>
-      <c r="AK16" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="AH16" t="inlineStr">
+        <is>
+          <t>Gabriel Martinelli</t>
+        </is>
+      </c>
+      <c r="AI16" t="n">
+        <v>1.39594077</v>
+      </c>
+      <c r="AJ16" t="inlineStr">
+        <is>
+          <t>+0.81</t>
+        </is>
+      </c>
+      <c r="AK16" t="n">
+        <v>5</v>
+      </c>
       <c r="AL16" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="AM16" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="AN16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO16" t="n">
         <v>0</v>
       </c>
       <c r="AP16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ16" t="n">
         <v>0</v>
       </c>
       <c r="AR16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS16" t="n">
         <v>1</v>
@@ -3520,10 +3538,10 @@
         <v>0</v>
       </c>
       <c r="AV16" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AW16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX16" t="n">
         <v>0</v>
@@ -3543,19 +3561,15 @@
       <c r="BC16" t="n">
         <v>0</v>
       </c>
-      <c r="BD16" t="inlineStr">
-        <is>
-          <t>GK</t>
-        </is>
-      </c>
+      <c r="BD16" t="inlineStr"/>
       <c r="BE16" t="n">
         <v>0</v>
       </c>
       <c r="BF16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BG16" t="n">
-        <v>3.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -3571,17 +3585,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>R. Doan</t>
+          <t>Z. Suzuki</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>RWB</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -3591,20 +3605,18 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>7o11dzx2cccrslutrjl16ik89</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>2</v>
-      </c>
+          <t>2mfunwzltzdnmzlcjyvx752i</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="K17" t="inlineStr"/>
@@ -3615,22 +3627,22 @@
         </is>
       </c>
       <c r="N17" t="n">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="n">
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>RWB</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="S17" t="n">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
@@ -3654,35 +3666,23 @@
         <v>1</v>
       </c>
       <c r="AE17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF17" t="n">
-        <v>-0.2</v>
+        <v>0</v>
       </c>
       <c r="AG17" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH17" t="inlineStr">
-        <is>
-          <t>R. Doan</t>
-        </is>
-      </c>
-      <c r="AI17" t="n">
-        <v>0.2264691699999999</v>
-      </c>
-      <c r="AJ17" t="inlineStr">
-        <is>
-          <t>-0.38</t>
-        </is>
-      </c>
-      <c r="AK17" t="n">
-        <v>17</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="AH17" t="inlineStr"/>
+      <c r="AI17" t="inlineStr"/>
+      <c r="AJ17" t="inlineStr"/>
+      <c r="AK17" t="inlineStr"/>
       <c r="AL17" t="n">
         <v>0</v>
       </c>
       <c r="AM17" t="n">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="AN17" t="n">
         <v>0</v>
@@ -3697,19 +3697,19 @@
         <v>0</v>
       </c>
       <c r="AR17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AS17" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AT17" t="n">
         <v>0</v>
       </c>
       <c r="AU17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AV17" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AW17" t="n">
         <v>0</v>
@@ -3732,7 +3732,11 @@
       <c r="BC17" t="n">
         <v>0</v>
       </c>
-      <c r="BD17" t="inlineStr"/>
+      <c r="BD17" t="inlineStr">
+        <is>
+          <t>GK</t>
+        </is>
+      </c>
       <c r="BE17" t="n">
         <v>0</v>
       </c>
@@ -3740,7 +3744,7 @@
         <v>0</v>
       </c>
       <c r="BG17" t="n">
-        <v>0</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="18">
@@ -3756,17 +3760,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>K. Nakamura</t>
+          <t>R. Doan</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 13</t>
+          <t xml:space="preserve"> 10</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>LWB</t>
+          <t>RWB</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -3776,12 +3780,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>8wq90yejo2ktnfuzrkju45all</t>
+          <t>7o11dzx2cccrslutrjl16ik89</t>
         </is>
       </c>
       <c r="I18" t="n">
@@ -3811,7 +3815,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>LWB</t>
+          <t>RWB</t>
         </is>
       </c>
       <c r="S18" t="n">
@@ -3849,19 +3853,19 @@
       </c>
       <c r="AH18" t="inlineStr">
         <is>
-          <t>K. Nakamura</t>
+          <t>R. Doan</t>
         </is>
       </c>
       <c r="AI18" t="n">
-        <v>-0.04520977000000001</v>
+        <v>0.2264691699999999</v>
       </c>
       <c r="AJ18" t="inlineStr">
         <is>
-          <t>-0.65</t>
+          <t>-0.36</t>
         </is>
       </c>
       <c r="AK18" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="AL18" t="n">
         <v>0</v>
@@ -3882,16 +3886,16 @@
         <v>0</v>
       </c>
       <c r="AR18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AS18" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AT18" t="n">
         <v>0</v>
       </c>
       <c r="AU18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AV18" t="n">
         <v>0</v>
@@ -3941,17 +3945,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>H. Ito</t>
+          <t>K. Nakamura</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 21</t>
+          <t xml:space="preserve"> 13</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>LCB(3)</t>
+          <t>LWB</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -3961,18 +3965,20 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>8p2yagsx6ujdbmeonkd3u4c89</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr"/>
+          <t>8wq90yejo2ktnfuzrkju45all</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>2</v>
+      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K19" t="inlineStr"/>
@@ -3983,22 +3989,22 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>95</v>
+        <v>65</v>
       </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="n">
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>95</v>
+        <v>65</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>LCB(3)</t>
+          <t>LWB</t>
         </is>
       </c>
       <c r="S19" t="n">
-        <v>95</v>
+        <v>65</v>
       </c>
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
@@ -4022,35 +4028,35 @@
         <v>1</v>
       </c>
       <c r="AE19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AF19" t="n">
-        <v>-0.4</v>
+        <v>-0.2</v>
       </c>
       <c r="AG19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>H. Ito</t>
+          <t>K. Nakamura</t>
         </is>
       </c>
       <c r="AI19" t="n">
-        <v>0.3033443199999999</v>
+        <v>-0.03886794000000002</v>
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
-          <t>-0.30</t>
+          <t>-0.63</t>
         </is>
       </c>
       <c r="AK19" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="AL19" t="n">
         <v>0</v>
       </c>
       <c r="AM19" t="n">
-        <v>95</v>
+        <v>65</v>
       </c>
       <c r="AN19" t="n">
         <v>0</v>
@@ -4065,16 +4071,16 @@
         <v>0</v>
       </c>
       <c r="AR19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS19" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AT19" t="n">
         <v>0</v>
       </c>
       <c r="AU19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV19" t="n">
         <v>0</v>
@@ -4124,17 +4130,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>S. Taniguchi</t>
+          <t>H. Ito</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 3</t>
+          <t xml:space="preserve"> 21</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>CB(3)</t>
+          <t>LCB(3)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -4144,12 +4150,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>954ldw96u7zxzmzdb7fqah80l</t>
+          <t>8p2yagsx6ujdbmeonkd3u4c89</t>
         </is>
       </c>
       <c r="I20" t="inlineStr"/>
@@ -4166,22 +4172,22 @@
         </is>
       </c>
       <c r="N20" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="n">
         <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>CB(3)</t>
+          <t>LCB(3)</t>
         </is>
       </c>
       <c r="S20" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
@@ -4215,25 +4221,25 @@
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>S. Taniguchi</t>
+          <t>H. Ito</t>
         </is>
       </c>
       <c r="AI20" t="n">
-        <v>0.83016494</v>
+        <v>0.29134432</v>
       </c>
       <c r="AJ20" t="inlineStr">
         <is>
-          <t>+0.22</t>
+          <t>-0.30</t>
         </is>
       </c>
       <c r="AK20" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="AL20" t="n">
         <v>0</v>
       </c>
       <c r="AM20" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="AN20" t="n">
         <v>0</v>
@@ -4248,10 +4254,10 @@
         <v>0</v>
       </c>
       <c r="AR20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AS20" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="AT20" t="n">
         <v>0</v>
@@ -4260,7 +4266,7 @@
         <v>0</v>
       </c>
       <c r="AV20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AW20" t="n">
         <v>0</v>
@@ -4307,17 +4313,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>T. Tomiyasu</t>
+          <t>S. Taniguchi</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 22</t>
+          <t xml:space="preserve"> 3</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>RCB(3)</t>
+          <t>CB(3)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -4327,12 +4333,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2922aevmtpw4qvcwohmxmqtbd</t>
+          <t>954ldw96u7zxzmzdb7fqah80l</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
@@ -4349,22 +4355,22 @@
         </is>
       </c>
       <c r="N21" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="n">
         <v>0</v>
       </c>
       <c r="Q21" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>RCB(3)</t>
+          <t>CB(3)</t>
         </is>
       </c>
       <c r="S21" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
@@ -4398,25 +4404,25 @@
       </c>
       <c r="AH21" t="inlineStr">
         <is>
-          <t>T. Tomiyasu</t>
+          <t>S. Taniguchi</t>
         </is>
       </c>
       <c r="AI21" t="n">
-        <v>1.15993392</v>
+        <v>0.89938688</v>
       </c>
       <c r="AJ21" t="inlineStr">
         <is>
-          <t>+0.55</t>
+          <t>+0.31</t>
         </is>
       </c>
       <c r="AK21" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="AL21" t="n">
         <v>0</v>
       </c>
       <c r="AM21" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="AN21" t="n">
         <v>0</v>
@@ -4431,10 +4437,10 @@
         <v>0</v>
       </c>
       <c r="AR21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AS21" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="AT21" t="n">
         <v>1</v>
@@ -4443,7 +4449,7 @@
         <v>0</v>
       </c>
       <c r="AV21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW21" t="n">
         <v>0</v>
@@ -4490,17 +4496,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>K. Sano</t>
+          <t>T. Tomiyasu</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 24</t>
+          <t xml:space="preserve"> 22</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>RDM(2)</t>
+          <t>RCB(3)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -4510,12 +4516,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>6dtp194pewnyuhwkxcn2xpf8q</t>
+          <t>2922aevmtpw4qvcwohmxmqtbd</t>
         </is>
       </c>
       <c r="I22" t="inlineStr"/>
@@ -4532,22 +4538,22 @@
         </is>
       </c>
       <c r="N22" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="n">
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>RDM(2)</t>
+          <t>RCB(3)</t>
         </is>
       </c>
       <c r="S22" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr"/>
@@ -4574,35 +4580,35 @@
         <v>2</v>
       </c>
       <c r="AF22" t="n">
-        <v>-0.1</v>
+        <v>-0.4</v>
       </c>
       <c r="AG22" t="n">
         <v>1</v>
       </c>
       <c r="AH22" t="inlineStr">
         <is>
-          <t>K. Sano</t>
+          <t>T. Tomiyasu</t>
         </is>
       </c>
       <c r="AI22" t="n">
-        <v>0.9468073599999999</v>
+        <v>1.16949594</v>
       </c>
       <c r="AJ22" t="inlineStr">
         <is>
-          <t>+0.34</t>
+          <t>+0.58</t>
         </is>
       </c>
       <c r="AK22" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AL22" t="n">
         <v>0</v>
       </c>
       <c r="AM22" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="AN22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO22" t="n">
         <v>0</v>
@@ -4611,13 +4617,13 @@
         <v>0</v>
       </c>
       <c r="AQ22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS22" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AT22" t="n">
         <v>1</v>
@@ -4626,13 +4632,13 @@
         <v>0</v>
       </c>
       <c r="AV22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AW22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AY22" t="n">
         <v>0</v>
@@ -4654,7 +4660,7 @@
         <v>0</v>
       </c>
       <c r="BF22" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BG22" t="n">
         <v>0</v>
@@ -4673,17 +4679,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>D. Kamada</t>
+          <t>K. Sano</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 15</t>
+          <t xml:space="preserve"> 24</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>LDM(2)</t>
+          <t>RDM(2)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -4693,20 +4699,18 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>az15xx7m923srf9gdbwmiyga1</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>2</v>
-      </c>
+          <t>6dtp194pewnyuhwkxcn2xpf8q</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="K23" t="inlineStr"/>
@@ -4717,25 +4721,35 @@
         </is>
       </c>
       <c r="N23" t="n">
-        <v>77</v>
-      </c>
-      <c r="O23" t="inlineStr"/>
+        <v>100</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
       <c r="P23" t="n">
         <v>0</v>
       </c>
       <c r="Q23" t="n">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>LDM(2)</t>
+          <t>RDM(2)</t>
         </is>
       </c>
       <c r="S23" t="n">
-        <v>77</v>
-      </c>
-      <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr"/>
+        <v>96.7</v>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="U23" t="n">
+        <v>3.3</v>
+      </c>
       <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr"/>
       <c r="X23" t="inlineStr"/>
@@ -4756,65 +4770,65 @@
         <v>1</v>
       </c>
       <c r="AE23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF23" t="n">
-        <v>-0.05</v>
+        <v>-0.1</v>
       </c>
       <c r="AG23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AH23" t="inlineStr">
         <is>
-          <t>D. Kamada</t>
+          <t>K. Sano</t>
         </is>
       </c>
       <c r="AI23" t="n">
-        <v>0.01904546000000001</v>
+        <v>0.9421268699999999</v>
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
-          <t>-0.59</t>
+          <t>+0.35</t>
         </is>
       </c>
       <c r="AK23" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="AL23" t="n">
         <v>0</v>
       </c>
       <c r="AM23" t="n">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="AN23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO23" t="n">
         <v>0</v>
       </c>
       <c r="AP23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AS23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AT23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU23" t="n">
         <v>0</v>
       </c>
       <c r="AV23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AW23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX23" t="n">
         <v>1</v>
@@ -4839,7 +4853,7 @@
         <v>0</v>
       </c>
       <c r="BF23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BG23" t="n">
         <v>0</v>
@@ -4858,17 +4872,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>A. Ueda</t>
+          <t>D. Kamada</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 18</t>
+          <t xml:space="preserve"> 15</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>LDM(2)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -4878,18 +4892,20 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>8d0ffyx2qnnp0limf5aou92ei</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr"/>
+          <t>az15xx7m923srf9gdbwmiyga1</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>2</v>
+      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K24" t="inlineStr"/>
@@ -4900,22 +4916,22 @@
         </is>
       </c>
       <c r="N24" t="n">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="n">
         <v>0</v>
       </c>
       <c r="Q24" t="n">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>LDM(2)</t>
         </is>
       </c>
       <c r="S24" t="n">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
@@ -4939,35 +4955,35 @@
         <v>1</v>
       </c>
       <c r="AE24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AF24" t="n">
-        <v>0</v>
+        <v>-0.05</v>
       </c>
       <c r="AG24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH24" t="inlineStr">
         <is>
-          <t>A. Ueda</t>
+          <t>D. Kamada</t>
         </is>
       </c>
       <c r="AI24" t="n">
-        <v>0.40641457</v>
+        <v>0.01904546000000001</v>
       </c>
       <c r="AJ24" t="inlineStr">
         <is>
-          <t>-0.20</t>
+          <t>-0.57</t>
         </is>
       </c>
       <c r="AK24" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="AL24" t="n">
         <v>0</v>
       </c>
       <c r="AM24" t="n">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="AN24" t="n">
         <v>0</v>
@@ -4976,7 +4992,7 @@
         <v>0</v>
       </c>
       <c r="AP24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ24" t="n">
         <v>0</v>
@@ -4985,7 +5001,7 @@
         <v>2</v>
       </c>
       <c r="AS24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT24" t="n">
         <v>0</v>
@@ -4997,10 +5013,10 @@
         <v>0</v>
       </c>
       <c r="AW24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY24" t="n">
         <v>0</v>
@@ -5041,17 +5057,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>J. Ito</t>
+          <t>A. Ueda</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 14</t>
+          <t xml:space="preserve"> 18</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>RAM(2)</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -5061,20 +5077,18 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>cmrdm4nnd62inlvsnc52vkicp</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>2</v>
-      </c>
+          <t>8d0ffyx2qnnp0limf5aou92ei</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="K25" t="inlineStr"/>
@@ -5085,25 +5099,35 @@
         </is>
       </c>
       <c r="N25" t="n">
-        <v>77</v>
-      </c>
-      <c r="O25" t="inlineStr"/>
+        <v>100</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>LCF(2)</t>
+        </is>
+      </c>
       <c r="P25" t="n">
         <v>0</v>
       </c>
       <c r="Q25" t="n">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>RAM(2)</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="S25" t="n">
-        <v>77</v>
-      </c>
-      <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr"/>
+        <v>96.7</v>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>LCF(2)</t>
+        </is>
+      </c>
+      <c r="U25" t="n">
+        <v>3.3</v>
+      </c>
       <c r="V25" t="inlineStr"/>
       <c r="W25" t="inlineStr"/>
       <c r="X25" t="inlineStr"/>
@@ -5124,35 +5148,35 @@
         <v>1</v>
       </c>
       <c r="AE25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF25" t="n">
-        <v>-0.05</v>
+        <v>0</v>
       </c>
       <c r="AG25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AH25" t="inlineStr">
         <is>
-          <t>J. Ito</t>
+          <t>A. Ueda</t>
         </is>
       </c>
       <c r="AI25" t="n">
-        <v>0.03070951999999999</v>
+        <v>0.36938632</v>
       </c>
       <c r="AJ25" t="inlineStr">
         <is>
-          <t>-0.57</t>
+          <t>-0.22</t>
         </is>
       </c>
       <c r="AK25" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="AL25" t="n">
         <v>0</v>
       </c>
       <c r="AM25" t="n">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="AN25" t="n">
         <v>0</v>
@@ -5161,28 +5185,28 @@
         <v>0</v>
       </c>
       <c r="AP25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AR25" t="n">
         <v>2</v>
       </c>
       <c r="AS25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AT25" t="n">
         <v>0</v>
       </c>
       <c r="AU25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV25" t="n">
         <v>0</v>
       </c>
       <c r="AW25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX25" t="n">
         <v>0</v>
@@ -5207,7 +5231,7 @@
         <v>0</v>
       </c>
       <c r="BF25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BG25" t="n">
         <v>0</v>
@@ -5226,17 +5250,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>D. Maeda</t>
+          <t>J. Ito</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 11</t>
+          <t xml:space="preserve"> 14</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>LAM(2)</t>
+          <t>RAM(2)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -5246,18 +5270,20 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>4x7o9h6ea8ldt9sxgz87vwycp</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr"/>
+          <t>cmrdm4nnd62inlvsnc52vkicp</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>2</v>
+      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K26" t="inlineStr"/>
@@ -5268,22 +5294,22 @@
         </is>
       </c>
       <c r="N26" t="n">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="n">
         <v>0</v>
       </c>
       <c r="Q26" t="n">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>LAM(2)</t>
+          <t>RAM(2)</t>
         </is>
       </c>
       <c r="S26" t="n">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr"/>
@@ -5307,35 +5333,35 @@
         <v>1</v>
       </c>
       <c r="AE26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AF26" t="n">
-        <v>-0.1</v>
+        <v>-0.05</v>
       </c>
       <c r="AG26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH26" t="inlineStr">
         <is>
-          <t>D. Maeda</t>
+          <t>J. Ito</t>
         </is>
       </c>
       <c r="AI26" t="n">
-        <v>0.37517091</v>
+        <v>0.02519200999999999</v>
       </c>
       <c r="AJ26" t="inlineStr">
         <is>
-          <t>-0.23</t>
+          <t>-0.56</t>
         </is>
       </c>
       <c r="AK26" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="AL26" t="n">
         <v>0</v>
       </c>
       <c r="AM26" t="n">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="AN26" t="n">
         <v>0</v>
@@ -5347,19 +5373,19 @@
         <v>1</v>
       </c>
       <c r="AQ26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AR26" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AS26" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AT26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AV26" t="n">
         <v>0</v>
@@ -5390,7 +5416,7 @@
         <v>0</v>
       </c>
       <c r="BF26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BG26" t="n">
         <v>0</v>
@@ -5409,68 +5435,66 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Y. Sugawara</t>
+          <t>D. Maeda</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 2</t>
+          <t xml:space="preserve"> 11</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>RWB</t>
+          <t>LAM(2)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>4x7o9h6ea8ldt9sxgz87vwycp</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>2</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
           <t>no</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>ad2qplv0aa66l11ipq6yh0hd5</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K27" t="n">
-        <v>65</v>
-      </c>
-      <c r="L27" t="n">
-        <v>2</v>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
       <c r="N27" t="n">
-        <v>30</v>
+        <v>96</v>
       </c>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="Q27" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>RWB</t>
+          <t>LAM(2)</t>
         </is>
       </c>
       <c r="S27" t="n">
-        <v>30</v>
+        <v>96</v>
       </c>
       <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr"/>
@@ -5491,38 +5515,38 @@
         </is>
       </c>
       <c r="AD27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF27" t="n">
-        <v>-0.2</v>
+        <v>-0.1</v>
       </c>
       <c r="AG27" t="n">
         <v>2</v>
       </c>
       <c r="AH27" t="inlineStr">
         <is>
-          <t>Y. Sugawara</t>
+          <t>D. Maeda</t>
         </is>
       </c>
       <c r="AI27" t="n">
-        <v>0.04879251999999998</v>
+        <v>0.37517091</v>
       </c>
       <c r="AJ27" t="inlineStr">
         <is>
-          <t>-0.56</t>
+          <t>-0.21</t>
         </is>
       </c>
       <c r="AK27" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="AL27" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="AM27" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="AN27" t="n">
         <v>0</v>
@@ -5531,22 +5555,22 @@
         <v>0</v>
       </c>
       <c r="AP27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ27" t="n">
         <v>1</v>
       </c>
       <c r="AR27" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AS27" t="n">
         <v>2</v>
       </c>
       <c r="AT27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AV27" t="n">
         <v>0</v>
@@ -5577,7 +5601,7 @@
         <v>0</v>
       </c>
       <c r="BF27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BG27" t="n">
         <v>0</v>
@@ -5596,17 +5620,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>S. Machino</t>
+          <t>Y. Sugawara</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 6</t>
+          <t xml:space="preserve"> 2</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>RAM(2)</t>
+          <t>RWB</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -5621,7 +5645,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>4o71xxq6qdkhug58a073fxega</t>
+          <t>ad2qplv0aa66l11ipq6yh0hd5</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
@@ -5631,7 +5655,7 @@
         </is>
       </c>
       <c r="K28" t="n">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="L28" t="n">
         <v>2</v>
@@ -5642,22 +5666,22 @@
         </is>
       </c>
       <c r="N28" t="n">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="n">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="Q28" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>RAM(2)</t>
+          <t>RWB</t>
         </is>
       </c>
       <c r="S28" t="n">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="T28" t="inlineStr"/>
       <c r="U28" t="inlineStr"/>
@@ -5684,18 +5708,18 @@
         <v>1</v>
       </c>
       <c r="AF28" t="n">
-        <v>-0.05</v>
+        <v>-0.2</v>
       </c>
       <c r="AG28" t="n">
         <v>2</v>
       </c>
       <c r="AH28" t="inlineStr">
         <is>
-          <t>S. Machino</t>
+          <t>Y. Sugawara</t>
         </is>
       </c>
       <c r="AI28" t="n">
-        <v>0.08388499000000001</v>
+        <v>0.06249598999999997</v>
       </c>
       <c r="AJ28" t="inlineStr">
         <is>
@@ -5703,13 +5727,13 @@
         </is>
       </c>
       <c r="AK28" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="AL28" t="n">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="AM28" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="AN28" t="n">
         <v>0</v>
@@ -5727,13 +5751,13 @@
         <v>0</v>
       </c>
       <c r="AS28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AT28" t="n">
         <v>0</v>
       </c>
       <c r="AU28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV28" t="n">
         <v>0</v>
@@ -5783,17 +5807,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>A. Tanaka</t>
+          <t>S. Machino</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 7</t>
+          <t xml:space="preserve"> 6</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>LDM(2)</t>
+          <t>RAM(2)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -5808,7 +5832,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>28ucbvor6b0yxreoieehudfc9</t>
+          <t>4o71xxq6qdkhug58a073fxega</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
@@ -5829,25 +5853,35 @@
         </is>
       </c>
       <c r="N29" t="n">
-        <v>18</v>
-      </c>
-      <c r="O29" t="inlineStr"/>
+        <v>23</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>RDM(2)</t>
+        </is>
+      </c>
       <c r="P29" t="n">
         <v>77</v>
       </c>
       <c r="Q29" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>LDM(2)</t>
+          <t>RAM(2)</t>
         </is>
       </c>
       <c r="S29" t="n">
-        <v>18</v>
-      </c>
-      <c r="T29" t="inlineStr"/>
-      <c r="U29" t="inlineStr"/>
+        <v>19.7</v>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>RDM(2)</t>
+        </is>
+      </c>
+      <c r="U29" t="n">
+        <v>3.3</v>
+      </c>
       <c r="V29" t="inlineStr"/>
       <c r="W29" t="inlineStr"/>
       <c r="X29" t="inlineStr"/>
@@ -5878,25 +5912,25 @@
       </c>
       <c r="AH29" t="inlineStr">
         <is>
-          <t>A. Tanaka</t>
+          <t>S. Machino</t>
         </is>
       </c>
       <c r="AI29" t="n">
-        <v>-0.68759959</v>
+        <v>0.0557195</v>
       </c>
       <c r="AJ29" t="inlineStr">
         <is>
-          <t>-1.29</t>
+          <t>-0.53</t>
         </is>
       </c>
       <c r="AK29" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="AL29" t="n">
         <v>77</v>
       </c>
       <c r="AM29" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="AN29" t="n">
         <v>0</v>
@@ -5908,10 +5942,10 @@
         <v>0</v>
       </c>
       <c r="AQ29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR29" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AS29" t="n">
         <v>0</v>
@@ -5920,7 +5954,7 @@
         <v>0</v>
       </c>
       <c r="AU29" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AV29" t="n">
         <v>0</v>
@@ -5951,7 +5985,7 @@
         <v>0</v>
       </c>
       <c r="BF29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG29" t="n">
         <v>0</v>
@@ -5970,17 +6004,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>J. Suzuki</t>
+          <t>A. Tanaka</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 25</t>
+          <t xml:space="preserve"> 7</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>LWB</t>
+          <t>LDM(2)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -5995,7 +6029,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>bdcpptlf4dznvgwq5st8hxwyc</t>
+          <t>28ucbvor6b0yxreoieehudfc9</t>
         </is>
       </c>
       <c r="I30" t="inlineStr"/>
@@ -6005,7 +6039,7 @@
         </is>
       </c>
       <c r="K30" t="n">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="L30" t="n">
         <v>2</v>
@@ -6016,25 +6050,35 @@
         </is>
       </c>
       <c r="N30" t="n">
-        <v>30</v>
-      </c>
-      <c r="O30" t="inlineStr"/>
+        <v>23</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>LDM(3)</t>
+        </is>
+      </c>
       <c r="P30" t="n">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="Q30" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>LWB</t>
+          <t>LDM(2)</t>
         </is>
       </c>
       <c r="S30" t="n">
-        <v>30</v>
-      </c>
-      <c r="T30" t="inlineStr"/>
-      <c r="U30" t="inlineStr"/>
+        <v>19.7</v>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>LDM(3)</t>
+        </is>
+      </c>
+      <c r="U30" t="n">
+        <v>3.3</v>
+      </c>
       <c r="V30" t="inlineStr"/>
       <c r="W30" t="inlineStr"/>
       <c r="X30" t="inlineStr"/>
@@ -6058,32 +6102,32 @@
         <v>1</v>
       </c>
       <c r="AF30" t="n">
-        <v>-0.2</v>
+        <v>-0.05</v>
       </c>
       <c r="AG30" t="n">
         <v>2</v>
       </c>
       <c r="AH30" t="inlineStr">
         <is>
-          <t>J. Suzuki</t>
+          <t>A. Tanaka</t>
         </is>
       </c>
       <c r="AI30" t="n">
-        <v>-0.07497056000000005</v>
+        <v>-0.56170698</v>
       </c>
       <c r="AJ30" t="inlineStr">
         <is>
-          <t>-0.68</t>
+          <t>-1.15</t>
         </is>
       </c>
       <c r="AK30" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="AL30" t="n">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="AM30" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="AN30" t="n">
         <v>0</v>
@@ -6098,25 +6142,25 @@
         <v>0</v>
       </c>
       <c r="AR30" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AS30" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AT30" t="n">
         <v>0</v>
       </c>
       <c r="AU30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AV30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AW30" t="n">
         <v>0</v>
       </c>
       <c r="AX30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AY30" t="n">
         <v>0</v>
@@ -6141,6 +6185,390 @@
         <v>0</v>
       </c>
       <c r="BG30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>3hsg9oklerq6uua8pos3dmdck</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>6duaxcbrofil112qfq4v895go</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>K. Ogawa</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 19</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LAM(2)</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>dgex06nxjy9fdvc12o8keg99l</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K31" t="n">
+        <v>96</v>
+      </c>
+      <c r="L31" t="n">
+        <v>2</v>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N31" t="n">
+        <v>4</v>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>RCF(2)</t>
+        </is>
+      </c>
+      <c r="P31" t="n">
+        <v>96</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>100</v>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>LAM(2)</t>
+        </is>
+      </c>
+      <c r="S31" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>RCF(2)</t>
+        </is>
+      </c>
+      <c r="U31" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="V31" t="inlineStr"/>
+      <c r="W31" t="inlineStr"/>
+      <c r="X31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr"/>
+      <c r="Z31" t="inlineStr"/>
+      <c r="AA31" t="inlineStr"/>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>6duaxcbrofil112qfq4v895go</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="AD31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH31" t="inlineStr">
+        <is>
+          <t>K. Ogawa</t>
+        </is>
+      </c>
+      <c r="AI31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ31" t="inlineStr">
+        <is>
+          <t>-0.59</t>
+        </is>
+      </c>
+      <c r="AK31" t="n">
+        <v>25</v>
+      </c>
+      <c r="AL31" t="n">
+        <v>96</v>
+      </c>
+      <c r="AM31" t="n">
+        <v>100</v>
+      </c>
+      <c r="AN31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD31" t="inlineStr"/>
+      <c r="BE31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>3hsg9oklerq6uua8pos3dmdck</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>6duaxcbrofil112qfq4v895go</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>J. Suzuki</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 25</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LWB</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>bdcpptlf4dznvgwq5st8hxwyc</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K32" t="n">
+        <v>65</v>
+      </c>
+      <c r="L32" t="n">
+        <v>2</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N32" t="n">
+        <v>35</v>
+      </c>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="n">
+        <v>65</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>100</v>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>LWB</t>
+        </is>
+      </c>
+      <c r="S32" t="n">
+        <v>35</v>
+      </c>
+      <c r="T32" t="inlineStr"/>
+      <c r="U32" t="inlineStr"/>
+      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="inlineStr"/>
+      <c r="X32" t="inlineStr"/>
+      <c r="Y32" t="inlineStr"/>
+      <c r="Z32" t="inlineStr"/>
+      <c r="AA32" t="inlineStr"/>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>6duaxcbrofil112qfq4v895go</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="AD32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="AG32" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH32" t="inlineStr">
+        <is>
+          <t>J. Suzuki</t>
+        </is>
+      </c>
+      <c r="AI32" t="n">
+        <v>-0.07497056000000005</v>
+      </c>
+      <c r="AJ32" t="inlineStr">
+        <is>
+          <t>-0.66</t>
+        </is>
+      </c>
+      <c r="AK32" t="n">
+        <v>27</v>
+      </c>
+      <c r="AL32" t="n">
+        <v>65</v>
+      </c>
+      <c r="AM32" t="n">
+        <v>100</v>
+      </c>
+      <c r="AN32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS32" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD32" t="inlineStr"/>
+      <c r="BE32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG32" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>